<commit_message>
feat(import): multi-seat titles, unit forms and member photos (#677)
Splits a title cell into one role per seat with explicit rules for the
named forms, reads unit codes, N/A, advisor markers and project names,
counts distinct unresolved unit names, and imports member and advisor
photos the way the dashboard and the Team page editor store them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/import/fixtures/files/roster.xlsx
+++ b/scripts/import/fixtures/files/roster.xlsx
@@ -316,6 +316,75 @@
   </si>
   <si>
     <t>Writer</t>
+  </si>
+  <si>
+    <t>Olga</t>
+  </si>
+  <si>
+    <t>Serra</t>
+  </si>
+  <si>
+    <t>olga.serra@example.com</t>
+  </si>
+  <si>
+    <t>Rita</t>
+  </si>
+  <si>
+    <t>Longo</t>
+  </si>
+  <si>
+    <t>rita.longo@example.com</t>
+  </si>
+  <si>
+    <t>Structures (STR) - Cavour</t>
+  </si>
+  <si>
+    <t>Design &amp; Manufacturing - N/A</t>
+  </si>
+  <si>
+    <t>Head of Department - Design and Manufacturing Division Lead Engineer (acting)</t>
+  </si>
+  <si>
+    <t>Ettore</t>
+  </si>
+  <si>
+    <t>Bassi</t>
+  </si>
+  <si>
+    <t>ettore.bassi@example.com</t>
+  </si>
+  <si>
+    <t>Cavour</t>
+  </si>
+  <si>
+    <t>Sofia</t>
+  </si>
+  <si>
+    <t>Marchi</t>
+  </si>
+  <si>
+    <t>sofia.marchi@example.com</t>
+  </si>
+  <si>
+    <t>SENIOR ADVISOR (Cavour)</t>
+  </si>
+  <si>
+    <t>Pietro</t>
+  </si>
+  <si>
+    <t>Rinaldi</t>
+  </si>
+  <si>
+    <t>pietro.rinaldi@example.com</t>
+  </si>
+  <si>
+    <t>Operations (OPS), Avionics Legacy</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Social Media Manager - Recruitment Coordinator</t>
   </si>
   <si>
     <t>Number</t>
@@ -1029,6 +1098,157 @@
         <v>33</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C18" t="s">
+        <v>100</v>
+      </c>
+      <c r="E18" t="s">
+        <v>101</v>
+      </c>
+      <c r="M18" t="s">
+        <v>48</v>
+      </c>
+      <c r="N18" t="s">
+        <v>79</v>
+      </c>
+      <c r="P18" t="s">
+        <v>98</v>
+      </c>
+      <c r="R18" t="s">
+        <v>31</v>
+      </c>
+      <c r="S18" t="s">
+        <v>32</v>
+      </c>
+      <c r="T18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" t="s">
+        <v>104</v>
+      </c>
+      <c r="M19" t="s">
+        <v>105</v>
+      </c>
+      <c r="N19" t="s">
+        <v>106</v>
+      </c>
+      <c r="P19" t="s">
+        <v>107</v>
+      </c>
+      <c r="R19" t="s">
+        <v>31</v>
+      </c>
+      <c r="S19" t="s">
+        <v>32</v>
+      </c>
+      <c r="T19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" t="s">
+        <v>109</v>
+      </c>
+      <c r="E20" t="s">
+        <v>110</v>
+      </c>
+      <c r="M20" t="s">
+        <v>111</v>
+      </c>
+      <c r="P20" t="s">
+        <v>72</v>
+      </c>
+      <c r="R20" t="s">
+        <v>31</v>
+      </c>
+      <c r="S20" t="s">
+        <v>32</v>
+      </c>
+      <c r="T20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="E21" t="s">
+        <v>114</v>
+      </c>
+      <c r="M21" t="s">
+        <v>115</v>
+      </c>
+      <c r="R21" t="s">
+        <v>31</v>
+      </c>
+      <c r="S21" t="s">
+        <v>32</v>
+      </c>
+      <c r="T21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" t="s">
+        <v>117</v>
+      </c>
+      <c r="E22" t="s">
+        <v>118</v>
+      </c>
+      <c r="M22" t="s">
+        <v>119</v>
+      </c>
+      <c r="N22" t="s">
+        <v>120</v>
+      </c>
+      <c r="P22" t="s">
+        <v>121</v>
+      </c>
+      <c r="R22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S22" t="s">
+        <v>32</v>
+      </c>
+      <c r="T22" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1038,7 +1258,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1050,25 +1270,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="G1" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="H1" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="K1" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2">
@@ -1079,7 +1299,7 @@
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
         <v>24</v>
@@ -1091,7 +1311,7 @@
         <v>43</v>
       </c>
       <c r="J2" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3">
@@ -1099,13 +1319,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C3" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="F3" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="H3" t="s">
         <v>38</v>
@@ -1114,7 +1334,7 @@
         <v>85</v>
       </c>
       <c r="J3" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -1122,19 +1342,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="E4" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="H4" t="s">
         <v>61</v>
       </c>
       <c r="J4" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5">
@@ -1142,19 +1362,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="E5" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="H5" t="s">
         <v>61</v>
       </c>
       <c r="J5" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6">
@@ -1212,7 +1432,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1224,25 +1444,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="G1" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="H1" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="J1" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="K1" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="M1" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2">
@@ -1250,13 +1470,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="F2" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="H2" t="s">
         <v>38</v>
@@ -1294,19 +1514,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="B3" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="D3" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="E3" t="s">
         <v>0</v>
@@ -1318,22 +1538,22 @@
         <v>2</v>
       </c>
       <c r="H3" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="I3" t="s">
         <v>4</v>
       </c>
       <c r="J3" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="K3" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="L3" t="s">
         <v>12</v>
       </c>
       <c r="M3" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4">
@@ -1347,13 +1567,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="F4" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="I4" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="K4" t="s">
         <v>38</v>
@@ -1362,7 +1582,7 @@
         <v>85</v>
       </c>
       <c r="M4" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5">
@@ -1396,13 +1616,13 @@
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="F6" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="H6" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="K6" t="s">
         <v>61</v>
@@ -1426,7 +1646,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1435,15 +1655,15 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
         <v>38</v>
@@ -1474,10 +1694,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
         <v>38</v>
@@ -1498,15 +1718,15 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B2">
         <v>16</v>

</xml_diff>